<commit_message>
chore: update news radar report 2026-10-06
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-10-06.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-10-06.xlsx
@@ -477,12 +477,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Challenges Facing Biosimilar Formulary Adoption</t>
+          <t>Biosimilars Facing Formulary Adoption Hurdles</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Managed Healthcare Executive discusses the factors causing biosimilars to lose ground on commercial formularies. This impacts self-funded employers seeking cost savings from lower-priced alternatives to expensive reference biologics and challenges PBM formulary management strategies.</t>
+          <t>Industry expert Christine Johnston discusses the market dynamics and rebate structures causing biosimilars to lose ground on commercial formularies. This trend directly impacts self-funded employers seeking cost-effective alternatives to high-priced biologic drugs through their PBM strategies.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -492,7 +492,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 20:37:26 GMT</t>
+          <t>Mon, 05 Oct 2026 23:25:24 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -507,27 +507,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Trade Association Seeks Supreme Court Review of Louisiana 340B Law</t>
+          <t>PhRMA Report Attributes $12.8 Billion in 2025 Employer Costs to 340B Program</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>A trade association has received an extension to petition the Supreme Court to review a Louisiana law impacting the 340B drug pricing program. The outcome of this legal battle could reshape 340B operations and manufacturer restrictions, which indirectly influence overall drug pricing and supply chain costs for self-funded plans.</t>
+          <t>A new report from PhRMA claims that commercial employers faced $12.8 billion in higher health care costs in 2025 due to the 340B drug pricing program. This highlights the ongoing financial impact of 340B on self-funded plans and underscores why employer advocacy groups and PBMs are closely monitoring program reform and litigation. The findings emphasize the pressure self-funded employers face regarding drug cost drivers tied to institutional pricing disparities.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Mealey's</t>
+          <t>PhRMA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 19:23:28 GMT</t>
+          <t>Tue, 06 Oct 2026 00:20:23 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE9ITG9XSDM3NTNrQXJDcmhWZld6emo2eGt3Tm5JZkNTSF9mMnRvM0I1TlM5bk14Z2l3MF9VNl9kRW43U3JmampTUWNPVkNWMFI1LXgwOEhyaXdSRHFR0gFiQVVfeXFMTW1jM2lacEtKZ0lrZWQ4dlFaekJSb3BhaGJMeVNhNEQ5b0VyWVE5cEY4dmthNmRWTGVFSGxaNkxRNUt0ZmVvNVNtanlHRUFFMlN4UUFrRjlOanN6X2R1U3hKLXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNUUY0QkFLZnRBaUJ2cUhoR0NLc0xna0JiS2NSdXlfSW1xN3NxS0w0azlZS196MWp3ZVUyS3hTbFc3SnFmVWt2YTJhd3k4R3N2Um8tOHBQLURmWXpLX2xpekYtZVZ6N2E5ci13RUV2TzNTVjhyNHdFSmZoeHpkYkRPd29EMy1uaWlNNDJUQmJXT0g?oc=5</t>
         </is>
       </c>
     </row>
@@ -537,27 +537,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Informa PBM Contracting Summit Highlights Evolving Employer Strategies</t>
+          <t>McKesson and CD&amp;R to Acquire Option Care Health for $5.8B</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The Informa PBM Contracting Summit focuses on emerging trends in PBM contracting, drug pricing strategies, and fiduciary oversight. For self-funded employers, the insights from this summit provide critical guidance on navigating contract renewals, evaluating pricing transparency, and managing specialty drug costs.</t>
+          <t>Clayton, Dubilier &amp; Rice and McKesson are acquiring infusion therapy provider Option Care Health in a $5.8 billion deal. This major consolidation in specialty and infusion services significantly impacts the specialty drug distribution and care management landscape relevant to high-cost employer health plan management.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Drug Channels</t>
+          <t>Fierce Healthcare</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 10:30:00 GMT</t>
+          <t>Tue, 06 Oct 2026 16:30:00 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE0xbC1ncUYyWkRsUnp4S2Y1YUgtZk9MRDNwTFZzTVAzZHBWZl9YME5UR1lQcWlyd28zZGRPdm9qVllCcXBuYUJyWkpwX0ZiUDNhUjFYRkFKNHNleG9uUFdLMnJHaEFEdVkzbEFLbzk3OEp1Rk0tREtnaVlhY1F2QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPZXhuRUJZVE1IZkp3VllGdzJXbmkxeWFDb0lWZzdmemxZNmdKUTJncmhBM2pNazhOTWdWMFFDclpOQ2QzS1N5ajR0NlZva1lYX0hnTzNTQ1VLXzVtUVRINjI3czFFeGFneHNIZ3N1a25PTW5QeU5VZzBFUGlCQ1VjMjFHdlg4Z3pxVnY4dy1nY0tLaHM5MFhFTThETDFoS3JhSzRydXJDd2ZaajVQeE5DRDJR?oc=5</t>
         </is>
       </c>
     </row>
@@ -567,27 +567,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>PBM Disclosure Rules Leave Benefits Brokers Searching for Transparency</t>
+          <t>Mark Cuban's Cost-Plus Enters New Jersey Benefits Market</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>New PBM disclosure regulations aimed at increasing pricing transparency are still leaving benefits brokers with significant unanswered questions regarding hidden fees and true net costs. For self-funded employers, broker confusion makes navigating complex PBM contracts and evaluating true value even more challenging.</t>
+          <t>Mark Cuban's transparent pharmacy benefits model is expanding into New Jersey, challenging traditional PBM pricing structures. This move offers self-funded employers alternative contracting options focused on transparent drug pricing and bypassing traditional spread pricing. The entry signals continued disruption in the PBM market as employers seek out cost-containment strategies.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Insurance Business</t>
+          <t>BenefitsPRO</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 19:05:59 GMT</t>
+          <t>Tue, 06 Oct 2026 15:24:27 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPQ1BlTm9GQ3B4UVhhUjJ1cHg4MFIwT0t6bUpsYXFuVjVqbjM5eHpmdFZWekg0Z3MyVS1XZWRySVZRZF9vcVdacXEtMzJPU2dTNjBzcldPUFF5SjBKR2ZaQmNSM25xUC1EODUtS0FfZ2dDMTRudWpWTEUtTmhNY2cwa1pvcHp2S2Q5MGd0bmF0YUJfT0JKbi0zbU5MYXFhdGI0a0pjQmhYQTY4MmxOSkVhcWg2LVFHVEJqRS1LYlhEQ1o3RkJVa1VaQ1JaV3V0YlVaMGtQNlJQVWg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOMHNxZVo2SWd0N3FxcEN3UnVad3ZMZDNFQ3B1aTZxYTRRblJBcThKU1MycUVjMG56OXowR0RZalpGS2txeDlGZG01RmYxZGxIVEhacXF6RXpjZEM1Y0cySUJHTWc4aDkwN3JrdVdScHY0YkFKcUFXWndKSUFSLUNzMjlfbjZnRnIxamE4?oc=5</t>
         </is>
       </c>
     </row>
@@ -597,27 +597,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bipartisan Congressional Pressure Mounts on Pharmacy Benefit Managers</t>
+          <t>The Disconnect Between Rising Manufacturer Rebates and Employer Pharmacy Costs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Lawmakers from both parties are increasingly targeting pharmacy benefit managers over pricing transparency, rebates, and business practices. This bipartisan scrutiny signals a high likelihood of federal legislative or regulatory changes that will impact how PBMs operate and how self-funded employers manage drug costs.</t>
+          <t>Despite increasing manufacturer rebates, self-funded employers continue to see overall pharmacy benefit costs climb. This persistent trend highlights the limitations of traditional rebate-focused PBM pricing models and underscores the urgent need for self-funded plans to demand greater transparency and true cost management.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>NPR</t>
+          <t>Insurance Business</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 09:00:00 GMT</t>
+          <t>Tue, 06 Oct 2026 11:07:24 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOQ2dzXzUxbXZEbmt2RVNpUEE3MldDejNUeGVuNVRZSlU0ZHhXUWVkc2NLOUhRTGV2YjQ2bmY3VUNrMTNRWlA1ZEg3WU96TC12SUdGVzQwRGpKY0lrbkE0bzBOeWo0Q1dYZ0Y0cUh3UmRkV1l2NnpaN1VRZTgtM3JWQktvbUJnYjJ2b3I3Q0RseHdoXzRCYmx6R3FHTFQ0cURxMnlrWGNOZkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQbkdwWTdpcTZlX0w4ZnVld18wRXVPa2pkcmo1VHFCZ3VzcklXZTdKVkpMZUZKQmNrOFctaXBvOFBMbF9qUFc0aVhnSGlNNGFtVUE0aFFNU050SVRLZGVVbVVhX2Nmc1BOSHBnekxLdXVEdkRIMGtEdTVDTjNJRVVsRzFweUFQVjhPY1RLQnUwRU12ZDYzNUxDZWlFSmlRa3gyMVZoTUdoMXJFNFNrS2NMcFVZTXVXMmM?oc=5</t>
         </is>
       </c>
     </row>
@@ -627,27 +627,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Pharmacy Cost Control Requires Broader Strategy Beyond Standard Discounts</t>
+          <t>Congressional PBM Reform Faces Hurdles Before Reaching Consumers</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>A new advisory warns self-funded employers that relying solely on traditional pharmaceutical discounts is insufficient for managing total pharmacy spend. The report highlights the need for comprehensive cost-management strategies to combat rising employer health plan expenditures. This emphasizes the ongoing shift among self-funded plans toward holistic pharmacy benefit oversight rather than just chasing headline discounts.</t>
+          <t>The article discusses ongoing legislative efforts surrounding pharmacy benefit manager (PBM) reform and the challenges Congress faces in passing impactful policy changes. For self-funded employers and PBMs, this signals continued uncertainty regarding federal oversight, transparency mandates, and drug pricing regulations.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>PR Newswire</t>
+          <t>ProMarket</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Mon, 05 Oct 2026 12:08:00 GMT</t>
+          <t>Tue, 06 Oct 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQd210cVZjMElkYUlJVC1fVW5Za0MzYlBPSXg2UnNqR0xTdXRYUEFBeE43Z3ItSENTbXVjUXVlUldoTzVqZE53TzNxRzBSYW9GUkhNdlBYbkQ2dUtUT1EtYVFTWTNrUGRWMU51UlMyb25nX0ZNWjc1V2hhcDAzTlpWczN3dVM5U2swMWdRRGlSRFZCNTNDZGw2TXJtRFlJbi1XYXg3YUNCWFh0X01ONkk1RXJDYUZMVGFlU2JXMERhb1ZXbzFBeHpmc2F2SVoycExxTF9DVw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNdHdiRVo1U3dMWnNDVnIxckNHWjlMNjBCemVqUkhXNVh3R08zZkdudl9HNDBHSGN0cnFmQ3RVano0WFUtRU1STk53MG80NTNWSldoeFQta1lxcVN4aDV3eHFlOEpOTmg3UGhtbkF0R2VxbkFVLXpKdE9id0Z6UjVOVDBJczFNa0hqZUVNb09qUUk5enE1cFBIYXJ5VEdza2xibFNMbQ?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>